<commit_message>
Improve data anonymization for realism
</commit_message>
<xml_diff>
--- a/Grupikaaslastele/andmed/Tasude ja tundide aruanne DATACORP PROJEKTBÜROO OÜ August 2026.xlsx
+++ b/Grupikaaslastele/andmed/Tasude ja tundide aruanne DATACORP PROJEKTBÜROO OÜ August 2026.xlsx
@@ -419,77 +419,77 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Tekst 26549</t>
+          <t>isik</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Tekst 26550</t>
+          <t>tasuliik</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Tekst 26576</t>
+          <t>Unnamed: 2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Tekst 26552</t>
+          <t>tunde</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Tekst 26553</t>
+          <t>summa</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Tekst 26554</t>
+          <t>konto</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Tekst 26555</t>
+          <t>osakond</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Tekst 26556</t>
+          <t>kulukoht</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Tekst 26557</t>
+          <t>projekt</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Tekst 26558</t>
+          <t>sotsmaks</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Tekst 26559</t>
+          <t>töötuskindlustusmakse</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Tekst 26551</t>
+          <t>arvestuskuu</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Tekst 26561</t>
+          <t>kokku</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Tekst 26577</t>
+          <t>Unnamed: 13</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Tekst 26578</t>
+          <t>PR kanne</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,13 +511,13 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>214.9257602480102</v>
+        <v>224.9423321376321</v>
       </c>
       <c r="E2" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F2" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -527,43 +527,43 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K2" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L2" t="n">
-        <v>178921.3231870601</v>
+        <v>254104.4071322185</v>
       </c>
       <c r="M2" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>6273.895102708872</v>
+        <v>4237.606608895474</v>
       </c>
       <c r="P2" t="n">
-        <v>157678.463932261</v>
+        <v>170270.1924888241</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F3" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -575,23 +575,23 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>178921.3231870601</v>
+        <v>254104.4071322185</v>
       </c>
       <c r="M3" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>6235.25247961716</v>
+        <v>4211.506039421847</v>
       </c>
       <c r="P3" t="n">
-        <v>157677.6856844022</v>
+        <v>170269.3520924287</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -601,13 +601,13 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>136.6647497229195</v>
+        <v>143.0339829353422</v>
       </c>
       <c r="E4" t="n">
-        <v>2127.52370119013</v>
+        <v>1317.631139127071</v>
       </c>
       <c r="F4" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -617,43 +617,43 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>588.5699803891274</v>
+        <v>520.7888721560862</v>
       </c>
       <c r="K4" t="n">
-        <v>16.32600936635679</v>
+        <v>10.12921929248831</v>
       </c>
       <c r="L4" t="n">
-        <v>178920.4400915936</v>
+        <v>254103.1529583393</v>
       </c>
       <c r="M4" t="n">
-        <v>2629.615788549779</v>
+        <v>2563.586760437222</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>6297.151073014555</v>
+        <v>4253.314498786888</v>
       </c>
       <c r="P4" t="n">
-        <v>157676.9074365433</v>
+        <v>170268.5116960332</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>688.5407746051135</v>
+        <v>426.4313317265809</v>
       </c>
       <c r="F5" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -663,43 +663,43 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>190.4782222093711</v>
+        <v>168.542300524961</v>
       </c>
       <c r="K5" t="n">
-        <v>5.28051934994923</v>
+        <v>3.276216329024409</v>
       </c>
       <c r="L5" t="n">
-        <v>178920.4400915936</v>
+        <v>254103.1529583393</v>
       </c>
       <c r="M5" t="n">
-        <v>851.0283498193894</v>
+        <v>829.6592300112836</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>6297.151073014555</v>
+        <v>4253.314498786888</v>
       </c>
       <c r="P5" t="n">
-        <v>157676.1291886845</v>
+        <v>170267.6712996378</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F6" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -711,23 +711,23 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>178920.4400915936</v>
+        <v>254103.1529583393</v>
       </c>
       <c r="M6" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>6706.732707879278</v>
+        <v>4529.960157404223</v>
       </c>
       <c r="P6" t="n">
-        <v>157675.3509408257</v>
+        <v>170266.8309032424</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -737,13 +737,13 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>186.8919654330523</v>
+        <v>195.602027945767</v>
       </c>
       <c r="E7" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F7" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -753,43 +753,43 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K7" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L7" t="n">
-        <v>178919.5569961271</v>
+        <v>254101.8987844602</v>
       </c>
       <c r="M7" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
-        <v>6234.196532857335</v>
+        <v>4210.792816313265</v>
       </c>
       <c r="P7" t="n">
-        <v>157674.5726929669</v>
+        <v>170265.990506847</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F8" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -801,23 +801,23 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>178919.5569961271</v>
+        <v>254101.8987844602</v>
       </c>
       <c r="M8" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
-        <v>6129.582378866045</v>
+        <v>4140.132784055777</v>
       </c>
       <c r="P8" t="n">
-        <v>157673.7944451081</v>
+        <v>170265.1501104515</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -827,13 +827,13 @@
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>196.2365637047049</v>
+        <v>205.3821293430554</v>
       </c>
       <c r="E9" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F9" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -843,43 +843,43 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K9" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L9" t="n">
-        <v>178918.6739006605</v>
+        <v>254100.644610581</v>
       </c>
       <c r="M9" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
-        <v>6519.892985363951</v>
+        <v>4403.762120941469</v>
       </c>
       <c r="P9" t="n">
-        <v>157604.530385673</v>
+        <v>170190.3548312583</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F10" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>178918.6739006605</v>
+        <v>254100.644610581</v>
       </c>
       <c r="M10" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>6640.371482342145</v>
+        <v>4485.137481330289</v>
       </c>
       <c r="P10" t="n">
-        <v>157603.7521378141</v>
+        <v>170189.5144348629</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Isik 36</t>
+          <t>Töötaja 37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -917,13 +917,13 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>74.75678617322093</v>
+        <v>78.24081117830681</v>
       </c>
       <c r="E11" t="n">
-        <v>189.3780666167318</v>
+        <v>117.2867956781399</v>
       </c>
       <c r="F11" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -933,29 +933,29 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>52.39024281471283</v>
+        <v>46.35685878749553</v>
       </c>
       <c r="K11" t="n">
-        <v>1.453353949527311</v>
+        <v>0.90171091624525</v>
       </c>
       <c r="L11" t="n">
-        <v>178917.790805194</v>
+        <v>254099.3904367019</v>
       </c>
       <c r="M11" t="n">
-        <v>234.0707000256974</v>
+        <v>228.1932403224128</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
-        <v>6140.10413408002</v>
+        <v>4147.239542887731</v>
       </c>
       <c r="P11" t="n">
-        <v>157602.9738899553</v>
+        <v>170188.6740384674</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -965,13 +965,13 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
-        <v>205.5811619763575</v>
+        <v>215.1622307403437</v>
       </c>
       <c r="E12" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F12" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -981,43 +981,43 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K12" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L12" t="n">
-        <v>178917.790805194</v>
+        <v>254099.3904367019</v>
       </c>
       <c r="M12" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
-        <v>5774.922546307011</v>
+        <v>3900.583217836059</v>
       </c>
       <c r="P12" t="n">
-        <v>157602.1956420965</v>
+        <v>170187.833642072</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F13" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1029,23 +1029,23 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>178917.790805194</v>
+        <v>254099.3904367019</v>
       </c>
       <c r="M13" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
-        <v>8119.815746831569</v>
+        <v>5484.405510211741</v>
       </c>
       <c r="P13" t="n">
-        <v>157601.4173942377</v>
+        <v>170186.9932456766</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1055,13 +1055,13 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>174.04314280953</v>
+        <v>182.1543885244955</v>
       </c>
       <c r="E14" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F14" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1071,43 +1071,43 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K14" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L14" t="n">
-        <v>178916.9077097275</v>
+        <v>254098.1362628227</v>
       </c>
       <c r="M14" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
-        <v>6658.812838254813</v>
+        <v>4497.593413476616</v>
       </c>
       <c r="P14" t="n">
-        <v>157600.6391463788</v>
+        <v>170186.1528492811</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F15" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1119,23 +1119,23 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
-        <v>178916.9077097275</v>
+        <v>254098.1362628227</v>
       </c>
       <c r="M15" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
-        <v>6616.398976735152</v>
+        <v>4468.945618615193</v>
       </c>
       <c r="P15" t="n">
-        <v>157599.86089852</v>
+        <v>170185.3124528857</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1145,13 +1145,13 @@
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
-        <v>168.2027688897471</v>
+        <v>176.0418251511903</v>
       </c>
       <c r="E16" t="n">
-        <v>2447.029749981438</v>
+        <v>1515.509601675516</v>
       </c>
       <c r="F16" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1161,43 +1161,43 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>676.956024378151</v>
+        <v>598.9961706882832</v>
       </c>
       <c r="K16" t="n">
-        <v>18.78459979764049</v>
+        <v>11.65461359246986</v>
       </c>
       <c r="L16" t="n">
-        <v>178916.0246142609</v>
+        <v>254096.8820889436</v>
       </c>
       <c r="M16" t="n">
-        <v>3024.526997995227</v>
+        <v>2948.5818431755</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
-        <v>6684.331551617264</v>
+        <v>4514.829638600709</v>
       </c>
       <c r="P16" t="n">
-        <v>157599.0826506612</v>
+        <v>170184.4720564903</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>302.7776529068308</v>
+        <v>187.51812893021</v>
       </c>
       <c r="F17" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1207,43 +1207,43 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>83.76088517891664</v>
+        <v>74.11478392812921</v>
       </c>
       <c r="K17" t="n">
-        <v>2.31325503633097</v>
+        <v>1.435223208357023</v>
       </c>
       <c r="L17" t="n">
-        <v>178916.0246142609</v>
+        <v>254096.8820889436</v>
       </c>
       <c r="M17" t="n">
-        <v>374.2215521536898</v>
+        <v>364.8249378288619</v>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>6684.331551617264</v>
+        <v>4514.829638600709</v>
       </c>
       <c r="P17" t="n">
-        <v>157598.3044028024</v>
+        <v>170183.6316600948</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F18" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1255,23 +1255,23 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>178916.0246142609</v>
+        <v>254096.8820889436</v>
       </c>
       <c r="M18" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
-        <v>6684.331551617264</v>
+        <v>4514.829638600709</v>
       </c>
       <c r="P18" t="n">
-        <v>157597.5261549436</v>
+        <v>170182.7912636994</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1281,13 +1281,13 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>179.8835167293129</v>
+        <v>188.2669518978008</v>
       </c>
       <c r="E19" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F19" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1297,43 +1297,43 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K19" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L19" t="n">
-        <v>178837.4291177399</v>
+        <v>253985.2606136996</v>
       </c>
       <c r="M19" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
-        <v>6684.331551617264</v>
+        <v>4514.829638600709</v>
       </c>
       <c r="P19" t="n">
-        <v>157596.7479070847</v>
+        <v>170181.950867304</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F20" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1345,23 +1345,23 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
-        <v>178837.4291177399</v>
+        <v>253985.2606136996</v>
       </c>
       <c r="M20" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
-        <v>6308.967620088793</v>
+        <v>4261.295805001985</v>
       </c>
       <c r="P20" t="n">
-        <v>157595.9696592259</v>
+        <v>170181.1104709085</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1371,13 +1371,13 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>93.44598271652616</v>
+        <v>97.80101397288351</v>
       </c>
       <c r="E21" t="n">
-        <v>1427.430864521395</v>
+        <v>884.0453128641232</v>
       </c>
       <c r="F21" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1387,43 +1387,43 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
-        <v>394.8848402862497</v>
+        <v>349.4089699720118</v>
       </c>
       <c r="K21" t="n">
-        <v>10.94859975310574</v>
+        <v>6.792888902380883</v>
       </c>
       <c r="L21" t="n">
-        <v>178836.5460222733</v>
+        <v>253984.0064398204</v>
       </c>
       <c r="M21" t="n">
-        <v>1764.288949531012</v>
+        <v>1719.988072895532</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
-        <v>5325.504062848391</v>
+        <v>3597.030368372296</v>
       </c>
       <c r="P21" t="n">
-        <v>157526.7055997908</v>
+        <v>170106.3151917153</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>686.1546109657427</v>
+        <v>424.9535181010363</v>
       </c>
       <c r="F22" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1433,43 +1433,43 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
-        <v>189.8220211882575</v>
+        <v>167.9616691623702</v>
       </c>
       <c r="K22" t="n">
-        <v>5.268408067036502</v>
+        <v>3.268702071389031</v>
       </c>
       <c r="L22" t="n">
-        <v>178836.5460222733</v>
+        <v>253984.0064398204</v>
       </c>
       <c r="M22" t="n">
-        <v>848.0893455141339</v>
+        <v>826.7940234063385</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>5508.371414219612</v>
+        <v>3720.545327426571</v>
       </c>
       <c r="P22" t="n">
-        <v>157525.927351932</v>
+        <v>170105.4747953199</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F23" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1481,37 +1481,37 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
-        <v>178836.5460222733</v>
+        <v>253984.0064398204</v>
       </c>
       <c r="M23" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>5525.693969398655</v>
+        <v>3732.245582707851</v>
       </c>
       <c r="P23" t="n">
-        <v>157525.1491040731</v>
+        <v>170104.6343989244</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tekst 26568</t>
+          <t>Lisatasu</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>713.7280574651389</v>
+        <v>442.0304755517735</v>
       </c>
       <c r="F24" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1521,29 +1521,29 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>197.4530040305622</v>
+        <v>174.7138500079832</v>
       </c>
       <c r="K24" t="n">
-        <v>5.486411159465598</v>
+        <v>3.403958708825819</v>
       </c>
       <c r="L24" t="n">
-        <v>178836.5460222733</v>
+        <v>253984.0064398204</v>
       </c>
       <c r="M24" t="n">
-        <v>882.1794629119971</v>
+        <v>860.0281460502056</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
-        <v>5542.563975966345</v>
+        <v>3743.640170942596</v>
       </c>
       <c r="P24" t="n">
-        <v>157524.3708562143</v>
+        <v>170103.794002529</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1553,13 +1553,13 @@
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
-        <v>168.2027688897471</v>
+        <v>176.0418251511903</v>
       </c>
       <c r="E25" t="n">
-        <v>2234.244554330879</v>
+        <v>1383.726158051559</v>
       </c>
       <c r="F25" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1569,43 +1569,43 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
-        <v>618.088442451801</v>
+        <v>546.9079184506973</v>
       </c>
       <c r="K25" t="n">
-        <v>17.14957660442227</v>
+        <v>10.64018881169395</v>
       </c>
       <c r="L25" t="n">
-        <v>178835.6629268068</v>
+        <v>253982.7522659413</v>
       </c>
       <c r="M25" t="n">
-        <v>2761.521100821361</v>
+        <v>2692.179961635354</v>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="n">
-        <v>5617.020793328808</v>
+        <v>3793.930890849001</v>
       </c>
       <c r="P25" t="n">
-        <v>157523.5926083555</v>
+        <v>170102.9536061336</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F26" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1617,37 +1617,37 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
-        <v>178835.6629268068</v>
+        <v>253982.7522659413</v>
       </c>
       <c r="M26" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
-        <v>5795.035817922735</v>
+        <v>3914.168419904309</v>
       </c>
       <c r="P26" t="n">
-        <v>157522.8143604967</v>
+        <v>170102.1132097382</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tekst 26568</t>
+          <t>Lisatasu</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>620.6171747119124</v>
+        <v>384.364467676688</v>
       </c>
       <c r="F27" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1657,29 +1657,29 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="n">
-        <v>171.6918220081357</v>
+        <v>151.9193865153035</v>
       </c>
       <c r="K27" t="n">
-        <v>4.759734184701943</v>
+        <v>2.953103250703194</v>
       </c>
       <c r="L27" t="n">
-        <v>178835.6629268068</v>
+        <v>253982.7522659413</v>
       </c>
       <c r="M27" t="n">
-        <v>767.0801236716579</v>
+        <v>747.8189238906695</v>
       </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
-        <v>5516.127594586426</v>
+        <v>3725.78412097414</v>
       </c>
       <c r="P27" t="n">
-        <v>157522.0361126379</v>
+        <v>170101.2728133427</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1689,13 +1689,13 @@
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="n">
-        <v>140.1689740747892</v>
+        <v>146.7015209593253</v>
       </c>
       <c r="E28" t="n">
-        <v>1946.503519913416</v>
+        <v>1205.520600698193</v>
       </c>
       <c r="F28" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1705,43 +1705,43 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
-        <v>538.4870250357494</v>
+        <v>476.4735881596359</v>
       </c>
       <c r="K28" t="n">
-        <v>14.93321183139312</v>
+        <v>9.265079664419945</v>
       </c>
       <c r="L28" t="n">
-        <v>178834.7798313403</v>
+        <v>253981.4980920621</v>
       </c>
       <c r="M28" t="n">
         <v>2062.87</v>
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
-        <v>5378.590529119147</v>
+        <v>3632.886811081185</v>
       </c>
       <c r="P28" t="n">
-        <v>157521.257864779</v>
+        <v>170100.4324169473</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F29" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1753,23 +1753,23 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
-        <v>178834.7798313403</v>
+        <v>253981.4980920621</v>
       </c>
       <c r="M29" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
-        <v>5135.936477870182</v>
+        <v>3468.989838879036</v>
       </c>
       <c r="P29" t="n">
-        <v>157520.4796169202</v>
+        <v>170099.5920205519</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1779,13 +1779,13 @@
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="n">
-        <v>149.5135723464419</v>
+        <v>156.4816223566136</v>
       </c>
       <c r="E30" t="n">
-        <v>2283.899483397786</v>
+        <v>1414.478755878367</v>
       </c>
       <c r="F30" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1795,43 +1795,43 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
-        <v>631.8263283454369</v>
+        <v>559.0637169771961</v>
       </c>
       <c r="K30" t="n">
-        <v>17.52502637471682</v>
+        <v>10.87313079839064</v>
       </c>
       <c r="L30" t="n">
-        <v>178833.8967358737</v>
+        <v>253980.243918183</v>
       </c>
       <c r="M30" t="n">
-        <v>2822.890309766812</v>
+        <v>2752.008204314803</v>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="n">
-        <v>5371.550884053642</v>
+        <v>3628.131990357297</v>
       </c>
       <c r="P30" t="n">
-        <v>157519.7013690614</v>
+        <v>170098.7516241565</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>588.4355285915091</v>
+        <v>364.4335315311162</v>
       </c>
       <c r="F31" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1841,43 +1841,43 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="n">
-        <v>162.7907726733532</v>
+        <v>144.0434030324179</v>
       </c>
       <c r="K31" t="n">
-        <v>4.517508526447391</v>
+        <v>2.802818097995652</v>
       </c>
       <c r="L31" t="n">
-        <v>178833.8967358737</v>
+        <v>253980.243918183</v>
       </c>
       <c r="M31" t="n">
-        <v>727.3102638267337</v>
+        <v>709.0476757840711</v>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
-        <v>4812.024809293687</v>
+        <v>3250.208650321156</v>
       </c>
       <c r="P31" t="n">
-        <v>157518.9231212026</v>
+        <v>170097.911227761</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>882.6532928872637</v>
+        <v>546.6502972966742</v>
       </c>
       <c r="F32" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1887,43 +1887,43 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
-        <v>244.1808670663111</v>
+        <v>216.0604220376383</v>
       </c>
       <c r="K32" t="n">
-        <v>6.770207148214722</v>
+        <v>4.20047001817579</v>
       </c>
       <c r="L32" t="n">
-        <v>178833.8967358737</v>
+        <v>253980.243918183</v>
       </c>
       <c r="M32" t="n">
-        <v>1090.953733024603</v>
+        <v>1063.560143808627</v>
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="n">
-        <v>4684.280392944313</v>
+        <v>3163.92563568518</v>
       </c>
       <c r="P32" t="n">
-        <v>157518.1448733438</v>
+        <v>170097.0708313656</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F33" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1935,10 +1935,10 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>178833.8967358737</v>
+        <v>253980.243918183</v>
       </c>
       <c r="M33" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
@@ -1947,7 +1947,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1957,13 +1957,13 @@
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="n">
-        <v>214.9257602480102</v>
+        <v>224.9423321376321</v>
       </c>
       <c r="E34" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F34" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1973,16 +1973,16 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K34" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L34" t="n">
-        <v>178833.0136404072</v>
+        <v>253978.9897443038</v>
       </c>
       <c r="M34" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
@@ -1991,21 +1991,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F35" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2017,10 +2017,10 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
-        <v>178833.0136404072</v>
+        <v>253978.9897443038</v>
       </c>
       <c r="M35" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
@@ -2029,7 +2029,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2039,13 +2039,13 @@
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="n">
-        <v>130.8243758031366</v>
+        <v>136.9214195620369</v>
       </c>
       <c r="E36" t="n">
-        <v>2103.586313569775</v>
+        <v>1302.806088153354</v>
       </c>
       <c r="F36" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2055,16 +2055,16 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="n">
-        <v>581.9444668533678</v>
+        <v>514.926368398314</v>
       </c>
       <c r="K36" t="n">
-        <v>16.14434012266588</v>
+        <v>10.01650542795765</v>
       </c>
       <c r="L36" t="n">
-        <v>178832.1305449407</v>
+        <v>253977.7355704247</v>
       </c>
       <c r="M36" t="n">
-        <v>2600.027479333775</v>
+        <v>2534.741406640613</v>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
@@ -2073,21 +2073,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>708.6906008931338</v>
+        <v>438.910646786735</v>
       </c>
       <c r="F37" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2097,16 +2097,16 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="n">
-        <v>196.0559308888365</v>
+        <v>173.4776671069833</v>
       </c>
       <c r="K37" t="n">
-        <v>5.437966027814689</v>
+        <v>3.373901678284311</v>
       </c>
       <c r="L37" t="n">
-        <v>178832.1305449407</v>
+        <v>253977.7355704247</v>
       </c>
       <c r="M37" t="n">
-        <v>875.9399101210779</v>
+        <v>853.9452669484372</v>
       </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
@@ -2115,21 +2115,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F38" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2141,10 +2141,10 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
-        <v>178832.1305449407</v>
+        <v>253977.7355704247</v>
       </c>
       <c r="M38" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
@@ -2153,7 +2153,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2163,13 +2163,13 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
-        <v>196.2365637047049</v>
+        <v>205.3821293430554</v>
       </c>
       <c r="E39" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F39" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2179,16 +2179,16 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K39" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L39" t="n">
-        <v>178831.2474494741</v>
+        <v>253976.4813965455</v>
       </c>
       <c r="M39" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
@@ -2197,21 +2197,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F40" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2223,10 +2223,10 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="n">
-        <v>178831.2474494741</v>
+        <v>253976.4813965455</v>
       </c>
       <c r="M40" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
@@ -2235,7 +2235,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2245,13 +2245,13 @@
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
-        <v>196.2365637047049</v>
+        <v>205.3821293430554</v>
       </c>
       <c r="E41" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F41" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2261,16 +2261,16 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K41" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L41" t="n">
-        <v>178830.3643540076</v>
+        <v>253975.2272226664</v>
       </c>
       <c r="M41" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
@@ -2279,21 +2279,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F42" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2305,10 +2305,10 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="n">
-        <v>178830.3643540076</v>
+        <v>253975.2272226664</v>
       </c>
       <c r="M42" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
@@ -2317,7 +2317,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2327,13 +2327,13 @@
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="n">
-        <v>196.2365637047049</v>
+        <v>205.3821293430554</v>
       </c>
       <c r="E43" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F43" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2343,16 +2343,16 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K43" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L43" t="n">
-        <v>178829.4812585411</v>
+        <v>253973.9730487872</v>
       </c>
       <c r="M43" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
@@ -2361,21 +2361,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F44" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2387,10 +2387,10 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="n">
-        <v>178829.4812585411</v>
+        <v>253973.9730487872</v>
       </c>
       <c r="M44" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
@@ -2399,7 +2399,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2409,13 +2409,13 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>177.5473671613997</v>
+        <v>185.8219265484787</v>
       </c>
       <c r="E45" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F45" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2425,16 +2425,16 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K45" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L45" t="n">
-        <v>178828.5981630746</v>
+        <v>253972.7188749081</v>
       </c>
       <c r="M45" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
@@ -2443,21 +2443,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F46" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2469,10 +2469,10 @@
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="n">
-        <v>178828.5981630746</v>
+        <v>253972.7188749081</v>
       </c>
       <c r="M46" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
@@ -2481,7 +2481,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2491,13 +2491,13 @@
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="n">
-        <v>205.5811619763575</v>
+        <v>215.1622307403437</v>
       </c>
       <c r="E47" t="n">
-        <v>2854.874354247232</v>
+        <v>1768.098444847958</v>
       </c>
       <c r="F47" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2507,16 +2507,16 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="n">
-        <v>789.7802644599367</v>
+        <v>698.8273049660008</v>
       </c>
       <c r="K47" t="n">
-        <v>21.90931078912421</v>
+        <v>13.59329206239715</v>
       </c>
       <c r="L47" t="n">
-        <v>178827.715067608</v>
+        <v>253971.4647010289</v>
       </c>
       <c r="M47" t="n">
-        <v>3528.612887208515</v>
+        <v>3440.010255393503</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
@@ -2525,21 +2525,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F48" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2551,10 +2551,10 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="n">
-        <v>178827.715067608</v>
+        <v>253971.4647010289</v>
       </c>
       <c r="M48" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
@@ -2563,7 +2563,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2573,13 +2573,13 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>121.479777531484</v>
+        <v>127.1413181647486</v>
       </c>
       <c r="E49" t="n">
-        <v>1789.319724621529</v>
+        <v>1108.172560285337</v>
       </c>
       <c r="F49" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2589,16 +2589,16 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="n">
-        <v>494.9978315558191</v>
+        <v>437.992712855026</v>
       </c>
       <c r="K49" t="n">
-        <v>13.73419482303309</v>
+        <v>8.521168158517613</v>
       </c>
       <c r="L49" t="n">
-        <v>178749.119571087</v>
+        <v>253859.8432257849</v>
       </c>
       <c r="M49" t="n">
-        <v>2211.589076989187</v>
+        <v>2156.056600353703</v>
       </c>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
@@ -2607,21 +2607,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F50" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2633,10 +2633,10 @@
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="n">
-        <v>178749.119571087</v>
+        <v>253859.8432257849</v>
       </c>
       <c r="M50" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
@@ -2645,21 +2645,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tekst 26568</t>
+          <t>Lisatasu</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>439.0036088264666</v>
+        <v>271.886430621352</v>
       </c>
       <c r="F51" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2669,16 +2669,16 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="n">
-        <v>121.4501083431979</v>
+        <v>107.4636271891942</v>
       </c>
       <c r="K51" t="n">
-        <v>3.36693664973827</v>
+        <v>2.088963622634829</v>
       </c>
       <c r="L51" t="n">
-        <v>178749.119571087</v>
+        <v>253859.8432257849</v>
       </c>
       <c r="M51" t="n">
-        <v>542.6078385000286</v>
+        <v>528.9830845042479</v>
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2697,13 +2697,13 @@
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="n">
-        <v>149.5135723464419</v>
+        <v>156.4816223566136</v>
       </c>
       <c r="E52" t="n">
-        <v>1827.296339580404</v>
+        <v>1131.692472378659</v>
       </c>
       <c r="F52" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2713,16 +2713,16 @@
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="n">
-        <v>505.5076317810737</v>
+        <v>447.2921796784569</v>
       </c>
       <c r="K52" t="n">
-        <v>14.02486561293855</v>
+        <v>8.701510341766664</v>
       </c>
       <c r="L52" t="n">
-        <v>178748.2364756204</v>
+        <v>253858.5890519058</v>
       </c>
       <c r="M52" t="n">
-        <v>2258.531506864794</v>
+        <v>2201.820316960465</v>
       </c>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
@@ -2731,21 +2731,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>485.1866066720669</v>
+        <v>300.4887705273943</v>
       </c>
       <c r="F53" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2755,16 +2755,16 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="n">
-        <v>134.224860480038</v>
+        <v>118.7672087157613</v>
       </c>
       <c r="K53" t="n">
-        <v>3.730275137120098</v>
+        <v>2.314391351696142</v>
       </c>
       <c r="L53" t="n">
-        <v>178748.2364756204</v>
+        <v>253858.5890519058</v>
       </c>
       <c r="M53" t="n">
-        <v>599.696830858065</v>
+        <v>584.6385858185585</v>
       </c>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
@@ -2773,21 +2773,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
-        <v>80.86443444534449</v>
+        <v>50.08146175456572</v>
       </c>
       <c r="F54" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2797,16 +2797,16 @@
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="n">
-        <v>22.37433804248544</v>
+        <v>19.79765645995264</v>
       </c>
       <c r="K54" t="n">
-        <v>0.6176754285491071</v>
+        <v>0.3832271394042313</v>
       </c>
       <c r="L54" t="n">
-        <v>178748.2364756204</v>
+        <v>253858.5890519058</v>
       </c>
       <c r="M54" t="n">
-        <v>99.94947180967749</v>
+        <v>97.43976430309307</v>
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
@@ -2815,21 +2815,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F55" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2841,10 +2841,10 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="n">
-        <v>178748.2364756204</v>
+        <v>253858.5890519058</v>
       </c>
       <c r="M55" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
@@ -2853,7 +2853,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2863,13 +2863,13 @@
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="n">
-        <v>214.9257602480102</v>
+        <v>224.9423321376321</v>
       </c>
       <c r="E56" t="n">
-        <v>2398.321711247615</v>
+        <v>1485.343437827099</v>
       </c>
       <c r="F56" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2879,16 +2879,16 @@
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="n">
-        <v>663.4827356704482</v>
+        <v>587.0744977112162</v>
       </c>
       <c r="K56" t="n">
-        <v>18.40915002734594</v>
+        <v>11.42167160577317</v>
       </c>
       <c r="L56" t="n">
-        <v>178747.3533801539</v>
+        <v>253857.3348780266</v>
       </c>
       <c r="M56" t="n">
-        <v>2964.324060599479</v>
+        <v>2889.890587244045</v>
       </c>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
@@ -2897,21 +2897,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F57" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2923,10 +2923,10 @@
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="n">
-        <v>178747.3533801539</v>
+        <v>253857.3348780266</v>
       </c>
       <c r="M57" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2945,13 +2945,13 @@
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="n">
-        <v>149.5135723464419</v>
+        <v>156.4816223566136</v>
       </c>
       <c r="E58" t="n">
-        <v>1827.296339580404</v>
+        <v>1131.692472378659</v>
       </c>
       <c r="F58" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2961,16 +2961,16 @@
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="n">
-        <v>505.5076317810737</v>
+        <v>447.2921796784569</v>
       </c>
       <c r="K58" t="n">
-        <v>14.02486561293855</v>
+        <v>8.701510341766664</v>
       </c>
       <c r="L58" t="n">
-        <v>178746.4702846874</v>
+        <v>253856.0807041475</v>
       </c>
       <c r="M58" t="n">
-        <v>2258.531506864794</v>
+        <v>2201.820316960465</v>
       </c>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
@@ -2979,21 +2979,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>587.9683960271877</v>
+        <v>364.1442241017767</v>
       </c>
       <c r="F59" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="n">
-        <v>162.6637660241054</v>
+        <v>143.9310227686907</v>
       </c>
       <c r="K59" t="n">
-        <v>4.505397243534664</v>
+        <v>2.795303840360275</v>
       </c>
       <c r="L59" t="n">
-        <v>178746.4702846874</v>
+        <v>253856.0807041475</v>
       </c>
       <c r="M59" t="n">
-        <v>726.7271280518814</v>
+        <v>708.479182410074</v>
       </c>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
@@ -3021,21 +3021,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F60" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3047,10 +3047,10 @@
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="n">
-        <v>178746.4702846874</v>
+        <v>253856.0807041475</v>
       </c>
       <c r="M60" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
@@ -3059,7 +3059,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3069,13 +3069,13 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>196.2365637047049</v>
+        <v>205.3821293430554</v>
       </c>
       <c r="E61" t="n">
-        <v>2398.321711247615</v>
+        <v>1485.343437827099</v>
       </c>
       <c r="F61" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3085,16 +3085,16 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="n">
-        <v>663.4827356704482</v>
+        <v>587.0744977112162</v>
       </c>
       <c r="K61" t="n">
-        <v>18.40915002734594</v>
+        <v>11.42167160577317</v>
       </c>
       <c r="L61" t="n">
-        <v>178745.5871892208</v>
+        <v>253854.8265302683</v>
       </c>
       <c r="M61" t="n">
-        <v>2964.324060599479</v>
+        <v>2889.890587244045</v>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
@@ -3103,21 +3103,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F62" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3129,10 +3129,10 @@
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="n">
-        <v>178745.5871892208</v>
+        <v>253854.8265302683</v>
       </c>
       <c r="M62" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
@@ -3141,7 +3141,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3151,13 +3151,13 @@
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="n">
-        <v>121.479777531484</v>
+        <v>127.1413181647486</v>
       </c>
       <c r="E63" t="n">
-        <v>1355.568200842566</v>
+        <v>839.5388834641251</v>
       </c>
       <c r="F63" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3167,16 +3167,16 @@
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="n">
-        <v>375.0082996789707</v>
+        <v>331.8214586986953</v>
       </c>
       <c r="K63" t="n">
-        <v>10.403592022033</v>
+        <v>6.454747308788915</v>
       </c>
       <c r="L63" t="n">
-        <v>178744.7040937543</v>
+        <v>253853.5723563892</v>
       </c>
       <c r="M63" t="n">
-        <v>1675.477371021012</v>
+        <v>1633.406532035782</v>
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
@@ -3185,21 +3185,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tekst 26563</t>
+          <t>Põhipuhkuse tasu</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
-        <v>1221.539030495685</v>
+        <v>756.5311086028495</v>
       </c>
       <c r="F64" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3209,16 +3209,16 @@
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="n">
-        <v>337.9329419860538</v>
+        <v>299.0157867123121</v>
       </c>
       <c r="K64" t="n">
-        <v>9.374132974451156</v>
+        <v>5.816035409781863</v>
       </c>
       <c r="L64" t="n">
-        <v>178744.7040937543</v>
+        <v>253853.5723563892</v>
       </c>
       <c r="M64" t="n">
-        <v>1509.820160100982</v>
+        <v>1471.908934350702</v>
       </c>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
@@ -3227,21 +3227,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F65" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3253,10 +3253,10 @@
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="n">
-        <v>178744.7040937543</v>
+        <v>253853.5723563892</v>
       </c>
       <c r="M65" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
@@ -3265,7 +3265,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3275,13 +3275,13 @@
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="n">
-        <v>177.5473671613997</v>
+        <v>185.8219265484787</v>
       </c>
       <c r="E66" t="n">
-        <v>2398.321711247615</v>
+        <v>1485.343437827099</v>
       </c>
       <c r="F66" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3291,16 +3291,16 @@
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="n">
-        <v>663.4827356704482</v>
+        <v>587.0744977112162</v>
       </c>
       <c r="K66" t="n">
-        <v>18.40915002734594</v>
+        <v>11.42167160577317</v>
       </c>
       <c r="L66" t="n">
-        <v>178743.8209982878</v>
+        <v>253852.31818251</v>
       </c>
       <c r="M66" t="n">
-        <v>2964.324060599479</v>
+        <v>2889.890587244045</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
@@ -3309,21 +3309,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F67" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3335,10 +3335,10 @@
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="n">
-        <v>178743.8209982878</v>
+        <v>253852.31818251</v>
       </c>
       <c r="M67" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
@@ -3347,7 +3347,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3357,13 +3357,13 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>205.5811619763575</v>
+        <v>215.1622307403437</v>
       </c>
       <c r="E68" t="n">
-        <v>2398.321711247615</v>
+        <v>1485.343437827099</v>
       </c>
       <c r="F68" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3373,16 +3373,16 @@
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="n">
-        <v>663.4827356704482</v>
+        <v>587.0744977112162</v>
       </c>
       <c r="K68" t="n">
-        <v>18.40915002734594</v>
+        <v>11.42167160577317</v>
       </c>
       <c r="L68" t="n">
-        <v>178742.9379028213</v>
+        <v>253851.0640086309</v>
       </c>
       <c r="M68" t="n">
-        <v>2964.324060599479</v>
+        <v>2889.890587244045</v>
       </c>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
@@ -3391,21 +3391,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F69" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3417,10 +3417,10 @@
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="n">
-        <v>178742.9379028213</v>
+        <v>253851.0640086309</v>
       </c>
       <c r="M69" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
@@ -3429,7 +3429,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3439,13 +3439,13 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>158.8581706180945</v>
+        <v>166.261723753902</v>
       </c>
       <c r="E70" t="n">
-        <v>1853.253759911338</v>
+        <v>1147.768582506277</v>
       </c>
       <c r="F70" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3455,16 +3455,16 @@
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="n">
-        <v>512.694091351011</v>
+        <v>453.6510296010245</v>
       </c>
       <c r="K70" t="n">
-        <v>14.21864613954219</v>
+        <v>8.821738463932697</v>
       </c>
       <c r="L70" t="n">
-        <v>178742.0548073547</v>
+        <v>253849.8098347517</v>
       </c>
       <c r="M70" t="n">
-        <v>2290.615637197166</v>
+        <v>2233.098822397782</v>
       </c>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
@@ -3473,21 +3473,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F71" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3499,10 +3499,10 @@
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="n">
-        <v>178742.0548073547</v>
+        <v>253849.8098347517</v>
       </c>
       <c r="M71" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
@@ -3511,21 +3511,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tekst 26568</t>
+          <t>Lisatasu</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
-        <v>301.3636300094259</v>
+        <v>186.6423875224799</v>
       </c>
       <c r="F72" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3535,16 +3535,16 @@
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="n">
-        <v>83.36928134373596</v>
+        <v>73.76827811497016</v>
       </c>
       <c r="K72" t="n">
-        <v>2.31325503633097</v>
+        <v>1.435223208357023</v>
       </c>
       <c r="L72" t="n">
-        <v>178742.0548073547</v>
+        <v>253849.8098347517</v>
       </c>
       <c r="M72" t="n">
-        <v>372.4838075446301</v>
+        <v>363.1308275743507</v>
       </c>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
@@ -3553,7 +3553,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3563,13 +3563,13 @@
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
-        <v>186.8919654330523</v>
+        <v>195.602027945767</v>
       </c>
       <c r="E73" t="n">
-        <v>2398.321711247615</v>
+        <v>1485.343437827099</v>
       </c>
       <c r="F73" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3579,16 +3579,16 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="n">
-        <v>663.4827356704482</v>
+        <v>587.0744977112162</v>
       </c>
       <c r="K73" t="n">
-        <v>18.40915002734594</v>
+        <v>11.42167160577317</v>
       </c>
       <c r="L73" t="n">
-        <v>178741.1717118882</v>
+        <v>253848.5556608726</v>
       </c>
       <c r="M73" t="n">
-        <v>2964.324060599479</v>
+        <v>2889.890587244045</v>
       </c>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
@@ -3597,21 +3597,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F74" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3623,10 +3623,10 @@
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="n">
-        <v>178741.1717118882</v>
+        <v>253848.5556608726</v>
       </c>
       <c r="M74" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
@@ -3635,7 +3635,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3645,13 +3645,13 @@
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
-        <v>164.6985445378774</v>
+        <v>172.3742871272072</v>
       </c>
       <c r="E75" t="n">
-        <v>1999.28949968172</v>
+        <v>1238.212340213546</v>
       </c>
       <c r="F75" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3661,16 +3661,16 @@
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="n">
-        <v>553.0927896992451</v>
+        <v>489.397318488271</v>
       </c>
       <c r="K75" t="n">
-        <v>15.34499545042586</v>
+        <v>9.520564424022766</v>
       </c>
       <c r="L75" t="n">
-        <v>178740.2886164217</v>
+        <v>253847.3014869934</v>
       </c>
       <c r="M75" t="n">
-        <v>2471.119484944934</v>
+        <v>2409.070261384827</v>
       </c>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
@@ -3679,21 +3679,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F76" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3705,10 +3705,10 @@
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="n">
-        <v>178740.2886164217</v>
+        <v>253847.3014869934</v>
       </c>
       <c r="M76" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
@@ -3717,21 +3717,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tekst 26568</t>
+          <t>Lisatasu</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
-        <v>142.8668134556625</v>
+        <v>88.4811586595887</v>
       </c>
       <c r="F77" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3741,16 +3741,16 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="n">
-        <v>39.52023569093692</v>
+        <v>34.96899206313299</v>
       </c>
       <c r="K77" t="n">
-        <v>1.090015462145483</v>
+        <v>0.6762831871839375</v>
       </c>
       <c r="L77" t="n">
-        <v>178740.2886164217</v>
+        <v>253847.3014869934</v>
       </c>
       <c r="M77" t="n">
-        <v>176.5735126252646</v>
+        <v>172.1397936463044</v>
       </c>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
@@ -3759,7 +3759,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3769,13 +3769,13 @@
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
-        <v>177.5473671613997</v>
+        <v>185.8219265484787</v>
       </c>
       <c r="E78" t="n">
-        <v>2020.550343960558</v>
+        <v>1251.379737808345</v>
       </c>
       <c r="F78" t="n">
-        <v>4011.281217658579</v>
+        <v>4333.689443635607</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="n">
-        <v>558.9774311143926</v>
+        <v>494.6042707076342</v>
       </c>
       <c r="K78" t="n">
-        <v>15.50244212829132</v>
+        <v>9.618249773282669</v>
       </c>
       <c r="L78" t="n">
-        <v>178739.4055209551</v>
+        <v>253846.0473131143</v>
       </c>
       <c r="M78" t="n">
-        <v>2497.395582959777</v>
+        <v>2434.686572817133</v>
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
@@ -3803,21 +3803,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Isik 35</t>
+          <t>Töötaja 36</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Tekst 26575</t>
+          <t>Autokompensatsioon</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
-        <v>422.9443487773677</v>
+        <v>261.9405103478457</v>
       </c>
       <c r="F79" t="n">
-        <v>3798.368201859292</v>
+        <v>4103.663464674057</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3829,10 +3829,10 @@
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="n">
-        <v>178739.4055209551</v>
+        <v>253846.0473131143</v>
       </c>
       <c r="M79" t="n">
-        <v>390.7009691510147</v>
+        <v>380.8905605780184</v>
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>

</xml_diff>